<commit_message>
Fixed dependencies and app execution
</commit_message>
<xml_diff>
--- a/Reliance_Valuation_Model.xlsx
+++ b/Reliance_Valuation_Model.xlsx
@@ -1,22 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
   <workbookPr defaultThemeVersion="124226"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Downloads\Python Practice\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F4C47BF-DC3F-45FC-B6BB-00301A5FE188}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Historical_Data" sheetId="1" r:id="rId1"/>
     <sheet name="DCF_Model" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -53,20 +47,12 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -82,7 +68,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -90,54 +76,26 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -175,7 +133,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -209,7 +167,6 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -244,10 +201,9 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -420,35 +376,29 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:E104"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.42578125" bestFit="1" customWidth="1"/>
-  </cols>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:5">
+      <c r="A1" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+    <row r="2" spans="1:5">
+      <c r="A2" s="1">
         <v>45439</v>
       </c>
       <c r="B2">
@@ -458,14 +408,14 @@
         <v>22530.69921875</v>
       </c>
       <c r="D2">
-        <v>-3.3676754465106103E-2</v>
+        <v>-0.0336767544651061</v>
       </c>
       <c r="E2">
-        <v>-1.8573791893592321E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="2">
+        <v>-0.01857379189359232</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" s="1">
         <v>45446</v>
       </c>
       <c r="B3">
@@ -475,14 +425,14 @@
         <v>23290.150390625</v>
       </c>
       <c r="D3">
-        <v>2.764950572764446E-2</v>
+        <v>0.02764950572764446</v>
       </c>
       <c r="E3">
-        <v>3.3707394719600492E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
+        <v>0.03370739471960049</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" s="1">
         <v>45453</v>
       </c>
       <c r="B4">
@@ -492,14 +442,14 @@
         <v>23465.599609375</v>
       </c>
       <c r="D4">
-        <v>5.1704303652939654E-3</v>
+        <v>0.005170430365293965</v>
       </c>
       <c r="E4">
-        <v>7.5331938955887079E-3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
+        <v>0.007533193895588708</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" s="1">
         <v>45460</v>
       </c>
       <c r="B5">
@@ -509,14 +459,14 @@
         <v>23501.099609375</v>
       </c>
       <c r="D5">
-        <v>-1.580328386777341E-2</v>
+        <v>-0.01580328386777341</v>
       </c>
       <c r="E5">
-        <v>1.512852882131988E-3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+        <v>0.001512852882131988</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" s="1">
         <v>45467</v>
       </c>
       <c r="B6">
@@ -526,14 +476,14 @@
         <v>24010.599609375</v>
       </c>
       <c r="D6">
-        <v>7.6468197544887317E-2</v>
+        <v>0.07646819754488732</v>
       </c>
       <c r="E6">
-        <v>2.1679836623336168E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+        <v>0.02167983662333617</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5">
+      <c r="A7" s="1">
         <v>45474</v>
       </c>
       <c r="B7">
@@ -543,14 +493,14 @@
         <v>24323.849609375</v>
       </c>
       <c r="D7">
-        <v>1.483643556640701E-2</v>
+        <v>0.01483643556640701</v>
       </c>
       <c r="E7">
-        <v>1.304632142038176E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="2">
+        <v>0.01304632142038176</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="1">
         <v>45481</v>
       </c>
       <c r="B8">
@@ -560,14 +510,14 @@
         <v>24502.150390625</v>
       </c>
       <c r="D8">
-        <v>5.0987734472711646E-3</v>
+        <v>0.005098773447271165</v>
       </c>
       <c r="E8">
-        <v>7.3302862874664587E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="2">
+        <v>0.007330286287466459</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5">
+      <c r="A9" s="1">
         <v>45488</v>
       </c>
       <c r="B9">
@@ -577,14 +527,14 @@
         <v>24530.900390625</v>
       </c>
       <c r="D9">
-        <v>-2.603766141936836E-2</v>
+        <v>-0.02603766141936836</v>
       </c>
       <c r="E9">
-        <v>1.173366400158971E-3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="2">
+        <v>0.001173366400158971</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" s="1">
         <v>45495</v>
       </c>
       <c r="B10">
@@ -594,14 +544,14 @@
         <v>24834.849609375</v>
       </c>
       <c r="D10">
-        <v>-2.9659528257880648E-2</v>
+        <v>-0.02965952825788065</v>
       </c>
       <c r="E10">
-        <v>1.23904632080345E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="2">
+        <v>0.0123904632080345</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" s="1">
         <v>45502</v>
       </c>
       <c r="B11">
@@ -611,14 +561,14 @@
         <v>24717.69921875</v>
       </c>
       <c r="D11">
-        <v>-6.4280253724419154E-3</v>
+        <v>-0.006428025372441915</v>
       </c>
       <c r="E11">
-        <v>-4.7171773724281607E-3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="2">
+        <v>-0.004717177372428161</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" s="1">
         <v>45509</v>
       </c>
       <c r="B12">
@@ -628,14 +578,14 @@
         <v>24367.5</v>
       </c>
       <c r="D12">
-        <v>-1.6690794054902151E-2</v>
+        <v>-0.01669079405490215</v>
       </c>
       <c r="E12">
-        <v>-1.4167953726225041E-2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="2">
+        <v>-0.01416795372622504</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" s="1">
         <v>45516</v>
       </c>
       <c r="B13">
@@ -645,14 +595,14 @@
         <v>24541.150390625</v>
       </c>
       <c r="D13">
-        <v>2.645317286265048E-3</v>
+        <v>0.002645317286265048</v>
       </c>
       <c r="E13">
-        <v>7.126311300913013E-3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="2">
+        <v>0.007126311300913013</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" s="1">
         <v>45523</v>
       </c>
       <c r="B14">
@@ -662,14 +612,14 @@
         <v>24823.150390625</v>
       </c>
       <c r="D14">
-        <v>1.4730734616668959E-2</v>
+        <v>0.01473073461666896</v>
       </c>
       <c r="E14">
-        <v>1.1490903870086109E-2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="2">
+        <v>0.01149090387008611</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" s="1">
         <v>45530</v>
       </c>
       <c r="B15">
@@ -679,14 +629,14 @@
         <v>25235.900390625</v>
       </c>
       <c r="D15">
-        <v>9.8493004641273529E-3</v>
+        <v>0.009849300464127353</v>
       </c>
       <c r="E15">
-        <v>1.6627623549180241E-2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="2">
+        <v>0.01662762354918024</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" s="1">
         <v>45537</v>
       </c>
       <c r="B16">
@@ -696,14 +646,14 @@
         <v>24852.150390625</v>
       </c>
       <c r="D16">
-        <v>-2.9676351493259309E-2</v>
+        <v>-0.02967635149325931</v>
       </c>
       <c r="E16">
-        <v>-1.520651112343752E-2</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="2">
+        <v>-0.01520651112343752</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" s="1">
         <v>45544</v>
       </c>
       <c r="B17">
@@ -713,14 +663,14 @@
         <v>25356.5</v>
       </c>
       <c r="D17">
-        <v>5.3249175250227321E-3</v>
+        <v>0.005324917525022732</v>
       </c>
       <c r="E17">
-        <v>2.0294002790408609E-2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="2">
+        <v>0.02029400279040861</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" s="1">
         <v>45551</v>
       </c>
       <c r="B18">
@@ -730,14 +680,14 @@
         <v>25790.94921875</v>
       </c>
       <c r="D18">
-        <v>9.0315597339958309E-3</v>
+        <v>0.009031559733995831</v>
       </c>
       <c r="E18">
-        <v>1.7133643000808441E-2</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="2">
+        <v>0.01713364300080844</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" s="1">
         <v>45558</v>
       </c>
       <c r="B19">
@@ -747,14 +697,14 @@
         <v>26178.94921875</v>
       </c>
       <c r="D19">
-        <v>2.7087475333576579E-2</v>
+        <v>0.02708747533357658</v>
       </c>
       <c r="E19">
-        <v>1.5044037220542711E-2</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="2">
+        <v>0.01504403722054271</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" s="1">
         <v>45565</v>
       </c>
       <c r="B20">
@@ -764,14 +714,14 @@
         <v>25014.599609375</v>
       </c>
       <c r="D20">
-        <v>-9.1503274272203505E-2</v>
+        <v>-0.09150327427220351</v>
       </c>
       <c r="E20">
-        <v>-4.4476560141728849E-2</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="2">
+        <v>-0.04447656014172885</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" s="1">
         <v>45572</v>
       </c>
       <c r="B21">
@@ -781,14 +731,14 @@
         <v>24964.25</v>
       </c>
       <c r="D21">
-        <v>-1.04037494511956E-2</v>
+        <v>-0.0104037494511956</v>
       </c>
       <c r="E21">
-        <v>-2.012808926037279E-3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="2">
+        <v>-0.002012808926037279</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" s="1">
         <v>45579</v>
       </c>
       <c r="B22">
@@ -798,14 +748,14 @@
         <v>24854.05078125</v>
       </c>
       <c r="D22">
-        <v>-9.3287239933012023E-3</v>
+        <v>-0.009328723993301202</v>
       </c>
       <c r="E22">
-        <v>-4.4142811720760946E-3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="2">
+        <v>-0.004414281172076095</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" s="1">
         <v>45586</v>
       </c>
       <c r="B23">
@@ -815,14 +765,14 @@
         <v>24180.80078125</v>
       </c>
       <c r="D23">
-        <v>-2.3136952557138431E-2</v>
+        <v>-0.02313695255713843</v>
       </c>
       <c r="E23">
-        <v>-2.708813971314095E-2</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="2">
+        <v>-0.02708813971314095</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" s="1">
         <v>45593</v>
       </c>
       <c r="B24">
@@ -832,14 +782,14 @@
         <v>24304.349609375</v>
       </c>
       <c r="D24">
-        <v>8.133481317738056E-3</v>
+        <v>0.008133481317738056</v>
       </c>
       <c r="E24">
-        <v>5.1093770319137199E-3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="2">
+        <v>0.00510937703191372</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" s="1">
         <v>45600</v>
       </c>
       <c r="B25">
@@ -849,14 +799,14 @@
         <v>24148.19921875</v>
       </c>
       <c r="D25">
-        <v>-4.1011492047175253E-2</v>
+        <v>-0.04101149204717525</v>
       </c>
       <c r="E25">
-        <v>-6.424791987223899E-3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="2">
+        <v>-0.006424791987223899</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5">
+      <c r="A26" s="1">
         <v>45607</v>
       </c>
       <c r="B26">
@@ -866,14 +816,14 @@
         <v>23532.69921875</v>
       </c>
       <c r="D26">
-        <v>-1.258028315040749E-2</v>
+        <v>-0.01258028315040749</v>
       </c>
       <c r="E26">
-        <v>-2.5488443027341431E-2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="2">
+        <v>-0.02548844302734143</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5">
+      <c r="A27" s="1">
         <v>45614</v>
       </c>
       <c r="B27">
@@ -883,14 +833,14 @@
         <v>23907.25</v>
       </c>
       <c r="D27">
-        <v>-1.7355915973427121E-3</v>
+        <v>-0.001735591597342712</v>
       </c>
       <c r="E27">
-        <v>1.591618444481591E-2</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="2">
+        <v>0.01591618444481591</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5">
+      <c r="A28" s="1">
         <v>45621</v>
       </c>
       <c r="B28">
@@ -900,14 +850,14 @@
         <v>24131.099609375</v>
       </c>
       <c r="D28">
-        <v>2.1179050297726269E-2</v>
+        <v>0.02117905029772627</v>
       </c>
       <c r="E28">
-        <v>9.3632521254012335E-3</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="2">
+        <v>0.009363252125401234</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5">
+      <c r="A29" s="1">
         <v>45628</v>
       </c>
       <c r="B29">
@@ -917,14 +867,14 @@
         <v>24677.80078125</v>
       </c>
       <c r="D29">
-        <v>1.497449825448482E-2</v>
+        <v>0.01497449825448482</v>
       </c>
       <c r="E29">
-        <v>2.2655460411037609E-2</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="2">
+        <v>0.02265546041103761</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5">
+      <c r="A30" s="1">
         <v>45635</v>
       </c>
       <c r="B30">
@@ -934,14 +884,14 @@
         <v>24768.30078125</v>
       </c>
       <c r="D30">
-        <v>-2.950704841957796E-2</v>
+        <v>-0.02950704841957796</v>
       </c>
       <c r="E30">
-        <v>3.667263578396307E-3</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="2">
+        <v>0.003667263578396307</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5">
+      <c r="A31" s="1">
         <v>45642</v>
       </c>
       <c r="B31">
@@ -951,14 +901,14 @@
         <v>23587.5</v>
       </c>
       <c r="D31">
-        <v>-5.3069853302249559E-2</v>
+        <v>-0.05306985330224956</v>
       </c>
       <c r="E31">
-        <v>-4.7673871198458888E-2</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="2">
+        <v>-0.04767387119845889</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5">
+      <c r="A32" s="1">
         <v>45649</v>
       </c>
       <c r="B32">
@@ -968,14 +918,14 @@
         <v>23813.400390625</v>
       </c>
       <c r="D32">
-        <v>1.3067311740050821E-2</v>
+        <v>0.01306731174005082</v>
       </c>
       <c r="E32">
-        <v>9.5771230789614137E-3</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="2">
+        <v>0.009577123078961414</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5">
+      <c r="A33" s="1">
         <v>45656</v>
       </c>
       <c r="B33">
@@ -985,14 +935,14 @@
         <v>24004.75</v>
       </c>
       <c r="D33">
-        <v>2.4650882545918851E-2</v>
+        <v>0.02465088254591885</v>
       </c>
       <c r="E33">
-        <v>8.0353753028203911E-3</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="2">
+        <v>0.008035375302820391</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5">
+      <c r="A34" s="1">
         <v>45663</v>
       </c>
       <c r="B34">
@@ -1002,14 +952,14 @@
         <v>23431.5</v>
       </c>
       <c r="D34">
-        <v>-7.3932407706446268E-3</v>
+        <v>-0.007393240770644627</v>
       </c>
       <c r="E34">
-        <v>-2.3880690280048689E-2</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="2">
+        <v>-0.02388069028004869</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5">
+      <c r="A35" s="1">
         <v>45670</v>
       </c>
       <c r="B35">
@@ -1019,14 +969,14 @@
         <v>23203.19921875</v>
       </c>
       <c r="D35">
-        <v>4.8675370619314373E-2</v>
+        <v>0.04867537061931437</v>
       </c>
       <c r="E35">
-        <v>-9.7433276252053558E-3</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="2">
+        <v>-0.009743327625205356</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5">
+      <c r="A36" s="1">
         <v>45677</v>
       </c>
       <c r="B36">
@@ -1036,14 +986,14 @@
         <v>23092.19921875</v>
       </c>
       <c r="D36">
-        <v>-4.3037488672091562E-2</v>
+        <v>-0.04303748867209156</v>
       </c>
       <c r="E36">
-        <v>-4.7838230820473893E-3</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="2">
+        <v>-0.004783823082047389</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5">
+      <c r="A37" s="1">
         <v>45684</v>
       </c>
       <c r="B37">
@@ -1053,14 +1003,14 @@
         <v>23482.150390625</v>
       </c>
       <c r="D37">
-        <v>1.468333996127091E-2</v>
+        <v>0.01468333996127091</v>
       </c>
       <c r="E37">
-        <v>1.688670568710382E-2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="2">
+        <v>0.01688670568710382</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5">
+      <c r="A38" s="1">
         <v>45691</v>
       </c>
       <c r="B38">
@@ -1070,14 +1020,14 @@
         <v>23559.94921875</v>
       </c>
       <c r="D38">
-        <v>1.6606269659071859E-3</v>
+        <v>0.001660626965907186</v>
       </c>
       <c r="E38">
-        <v>3.313104925691146E-3</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="2">
+        <v>0.003313104925691146</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5">
+      <c r="A39" s="1">
         <v>45698</v>
       </c>
       <c r="B39">
@@ -1087,14 +1037,14 @@
         <v>22929.25</v>
       </c>
       <c r="D39">
-        <v>-3.9038454449395799E-2</v>
+        <v>-0.0390384544493958</v>
       </c>
       <c r="E39">
-        <v>-2.6769973606227571E-2</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="2">
+        <v>-0.02676997360622757</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5">
+      <c r="A40" s="1">
         <v>45705</v>
       </c>
       <c r="B40">
@@ -1104,14 +1054,14 @@
         <v>22795.900390625</v>
       </c>
       <c r="D40">
-        <v>8.9546522347263569E-3</v>
+        <v>0.008954652234726357</v>
       </c>
       <c r="E40">
-        <v>-5.8156986981693359E-3</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="2">
+        <v>-0.005815698698169336</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5">
+      <c r="A41" s="1">
         <v>45712</v>
       </c>
       <c r="B41">
@@ -1121,14 +1071,14 @@
         <v>22124.69921875</v>
       </c>
       <c r="D41">
-        <v>-2.283927862558777E-2</v>
+        <v>-0.02283927862558777</v>
       </c>
       <c r="E41">
-        <v>-2.9443942128780209E-2</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="2">
+        <v>-0.02944394212878021</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5">
+      <c r="A42" s="1">
         <v>45719</v>
       </c>
       <c r="B42">
@@ -1138,14 +1088,14 @@
         <v>22552.5</v>
       </c>
       <c r="D42">
-        <v>4.1413341966133999E-2</v>
+        <v>0.041413341966134</v>
       </c>
       <c r="E42">
-        <v>1.9335891395416249E-2</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="2">
+        <v>0.01933589139541625</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5">
+      <c r="A43" s="1">
         <v>45726</v>
       </c>
       <c r="B43">
@@ -1155,14 +1105,14 @@
         <v>22397.19921875</v>
       </c>
       <c r="D43">
-        <v>-1.52025460023375E-3</v>
+        <v>-0.00152025460023375</v>
       </c>
       <c r="E43">
-        <v>-6.8861891697150623E-3</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A44" s="2">
+        <v>-0.006886189169715062</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5">
+      <c r="A44" s="1">
         <v>45733</v>
       </c>
       <c r="B44">
@@ -1172,14 +1122,14 @@
         <v>23350.400390625</v>
       </c>
       <c r="D44">
-        <v>2.2798174566797561E-2</v>
+        <v>0.02279817456679756</v>
       </c>
       <c r="E44">
-        <v>4.2558945096895062E-2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A45" s="2">
+        <v>0.04255894509689506</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5">
+      <c r="A45" s="1">
         <v>45740</v>
       </c>
       <c r="B45">
@@ -1189,14 +1139,14 @@
         <v>23519.349609375</v>
       </c>
       <c r="D45">
-        <v>-9.7932979427739486E-4</v>
+        <v>-0.0009793297942773949</v>
       </c>
       <c r="E45">
-        <v>7.2353885125597817E-3</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="2">
+        <v>0.007235388512559782</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5">
+      <c r="A46" s="1">
         <v>45747</v>
       </c>
       <c r="B46">
@@ -1206,14 +1156,14 @@
         <v>22904.44921875</v>
       </c>
       <c r="D46">
-        <v>-5.5211395237208187E-2</v>
+        <v>-0.05521139523720819</v>
       </c>
       <c r="E46">
-        <v>-2.614444705477292E-2</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A47" s="2">
+        <v>-0.02614444705477292</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5">
+      <c r="A47" s="1">
         <v>45754</v>
       </c>
       <c r="B47">
@@ -1223,14 +1173,14 @@
         <v>22828.55078125</v>
       </c>
       <c r="D47">
-        <v>1.182871036109856E-2</v>
+        <v>0.01182871036109856</v>
       </c>
       <c r="E47">
-        <v>-3.3136984336592512E-3</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A48" s="2">
+        <v>-0.003313698433659251</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5">
+      <c r="A48" s="1">
         <v>45761</v>
       </c>
       <c r="B48">
@@ -1240,14 +1190,14 @@
         <v>23851.650390625</v>
       </c>
       <c r="D48">
-        <v>4.5572076576162253E-2</v>
+        <v>0.04557207657616225</v>
       </c>
       <c r="E48">
-        <v>4.4816669230502093E-2</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A49" s="2">
+        <v>0.04481666923050209</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5">
+      <c r="A49" s="1">
         <v>45768</v>
       </c>
       <c r="B49">
@@ -1257,14 +1207,14 @@
         <v>24039.349609375</v>
       </c>
       <c r="D49">
-        <v>2.0321716029094938E-2</v>
+        <v>0.02032171602909494</v>
       </c>
       <c r="E49">
-        <v>7.8694436517390276E-3</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A50" s="2">
+        <v>0.007869443651739028</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5">
+      <c r="A50" s="1">
         <v>45775</v>
       </c>
       <c r="B50">
@@ -1274,14 +1224,14 @@
         <v>24346.69921875</v>
       </c>
       <c r="D50">
-        <v>9.1817916215070072E-2</v>
+        <v>0.09181791621507007</v>
       </c>
       <c r="E50">
-        <v>1.278527141412922E-2</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A51" s="2">
+        <v>0.01278527141412922</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5">
+      <c r="A51" s="1">
         <v>45782</v>
       </c>
       <c r="B51">
@@ -1291,14 +1241,14 @@
         <v>24008</v>
       </c>
       <c r="D51">
-        <v>-3.0004314298455181E-2</v>
+        <v>-0.03000431429845518</v>
       </c>
       <c r="E51">
-        <v>-1.391150462355728E-2</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="2">
+        <v>-0.01391150462355728</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5">
+      <c r="A52" s="1">
         <v>45789</v>
       </c>
       <c r="B52">
@@ -1308,14 +1258,14 @@
         <v>25019.80078125</v>
       </c>
       <c r="D52">
-        <v>5.7508038965779829E-2</v>
+        <v>0.05750803896577983</v>
       </c>
       <c r="E52">
-        <v>4.2144317779490237E-2</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A53" s="2">
+        <v>0.04214431777949024</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5">
+      <c r="A53" s="1">
         <v>45796</v>
       </c>
       <c r="B53">
@@ -1325,14 +1275,14 @@
         <v>24853.150390625</v>
       </c>
       <c r="D53">
-        <v>-2.0324036081353362E-2</v>
+        <v>-0.02032403608135336</v>
       </c>
       <c r="E53">
-        <v>-6.6607401106841824E-3</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A54" s="2">
+        <v>-0.006660740110684182</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5">
+      <c r="A54" s="1">
         <v>45803</v>
       </c>
       <c r="B54">
@@ -1342,14 +1292,14 @@
         <v>24750.69921875</v>
       </c>
       <c r="D54">
-        <v>-4.1351675206260374E-3</v>
+        <v>-0.004135167520626037</v>
       </c>
       <c r="E54">
-        <v>-4.1222609715364511E-3</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A55" s="2">
+        <v>-0.004122260971536451</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5">
+      <c r="A55" s="1">
         <v>45810</v>
       </c>
       <c r="B55">
@@ -1359,14 +1309,14 @@
         <v>25003.05078125</v>
       </c>
       <c r="D55">
-        <v>1.5905350048030401E-2</v>
+        <v>0.0159053500480304</v>
       </c>
       <c r="E55">
-        <v>1.0195734684894431E-2</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A56" s="2">
+        <v>0.01019573468489443</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5">
+      <c r="A56" s="1">
         <v>45817</v>
       </c>
       <c r="B56">
@@ -1376,14 +1326,14 @@
         <v>24718.599609375</v>
       </c>
       <c r="D56">
-        <v>-1.0806996130364181E-2</v>
+        <v>-0.01080699613036418</v>
       </c>
       <c r="E56">
-        <v>-1.1376658567134211E-2</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A57" s="2">
+        <v>-0.01137665856713421</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57" s="1">
         <v>45824</v>
       </c>
       <c r="B57">
@@ -1393,14 +1343,14 @@
         <v>25112.400390625</v>
       </c>
       <c r="D57">
-        <v>2.6822564067351399E-2</v>
+        <v>0.0268225640673514</v>
       </c>
       <c r="E57">
-        <v>1.5931354828881309E-2</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A58" s="2">
+        <v>0.01593135482888131</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58" s="1">
         <v>45831</v>
       </c>
       <c r="B58">
@@ -1410,14 +1360,14 @@
         <v>25637.80078125</v>
       </c>
       <c r="D58">
-        <v>3.355612525943874E-2</v>
+        <v>0.03355612525943874</v>
       </c>
       <c r="E58">
-        <v>2.092195020995069E-2</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="2">
+        <v>0.02092195020995069</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
+      <c r="A59" s="1">
         <v>45838</v>
       </c>
       <c r="B59">
@@ -1427,14 +1377,14 @@
         <v>25461</v>
       </c>
       <c r="D59">
-        <v>7.8527927686178334E-3</v>
+        <v>0.007852792768617833</v>
       </c>
       <c r="E59">
-        <v>-6.896097787736255E-3</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A60" s="2">
+        <v>-0.006896097787736255</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
+      <c r="A60" s="1">
         <v>45845</v>
       </c>
       <c r="B60">
@@ -1444,14 +1394,14 @@
         <v>25149.849609375</v>
       </c>
       <c r="D60">
-        <v>-2.1017550253890401E-2</v>
+        <v>-0.0210175502538904</v>
       </c>
       <c r="E60">
-        <v>-1.2220666534111021E-2</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="2">
+        <v>-0.01222066653411102</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61" s="1">
         <v>45852</v>
       </c>
       <c r="B61">
@@ -1461,14 +1411,14 @@
         <v>24968.400390625</v>
       </c>
       <c r="D61">
-        <v>-1.2841115043639941E-2</v>
+        <v>-0.01284111504363994</v>
       </c>
       <c r="E61">
-        <v>-7.2147238082235221E-3</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A62" s="2">
+        <v>-0.007214723808223522</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
+      <c r="A62" s="1">
         <v>45859</v>
       </c>
       <c r="B62">
@@ -1478,14 +1428,14 @@
         <v>24837</v>
       </c>
       <c r="D62">
-        <v>-5.7113868865755313E-2</v>
+        <v>-0.05711386886575531</v>
       </c>
       <c r="E62">
-        <v>-5.2626675545597301E-3</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A63" s="2">
+        <v>-0.00526266755455973</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5">
+      <c r="A63" s="1">
         <v>45866</v>
       </c>
       <c r="B63">
@@ -1495,14 +1445,14 @@
         <v>24565.349609375</v>
       </c>
       <c r="D63">
-        <v>1.437106912423491E-3</v>
+        <v>0.001437106912423491</v>
       </c>
       <c r="E63">
-        <v>-1.093732699702055E-2</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A64" s="2">
+        <v>-0.01093732699702055</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
+      <c r="A64" s="1">
         <v>45873</v>
       </c>
       <c r="B64">
@@ -1512,14 +1462,14 @@
         <v>24363.30078125</v>
       </c>
       <c r="D64">
-        <v>-1.858355936084544E-2</v>
+        <v>-0.01858355936084544</v>
       </c>
       <c r="E64">
-        <v>-8.2249522737462E-3</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A65" s="2">
+        <v>-0.0082249522737462</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5">
+      <c r="A65" s="1">
         <v>45880</v>
       </c>
       <c r="B65">
@@ -1529,14 +1479,14 @@
         <v>24631.30078125</v>
       </c>
       <c r="D65">
-        <v>4.3866534342182906E-3</v>
+        <v>0.004386653434218291</v>
       </c>
       <c r="E65">
-        <v>1.100015151502998E-2</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" s="2">
+        <v>0.01100015151502998</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5">
+      <c r="A66" s="1">
         <v>45887</v>
       </c>
       <c r="B66">
@@ -1546,14 +1496,14 @@
         <v>24870.099609375</v>
       </c>
       <c r="D66">
-        <v>2.9864664490100831E-2</v>
+        <v>0.02986466449010083</v>
       </c>
       <c r="E66">
-        <v>9.6949337043044093E-3</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A67" s="2">
+        <v>0.009694933704304409</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5">
+      <c r="A67" s="1">
         <v>45894</v>
       </c>
       <c r="B67">
@@ -1563,14 +1513,14 @@
         <v>24426.849609375</v>
       </c>
       <c r="D67">
-        <v>-3.6900370282270667E-2</v>
+        <v>-0.03690037028227067</v>
       </c>
       <c r="E67">
-        <v>-1.7822606542070799E-2</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="2">
+        <v>-0.0178226065420708</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5">
+      <c r="A68" s="1">
         <v>45901</v>
       </c>
       <c r="B68">
@@ -1580,14 +1530,14 @@
         <v>24741</v>
       </c>
       <c r="D68">
-        <v>1.3115273702121399E-2</v>
+        <v>0.0131152737021214</v>
       </c>
       <c r="E68">
-        <v>1.286086399387454E-2</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A69" s="2">
+        <v>0.01286086399387454</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5">
+      <c r="A69" s="1">
         <v>45908</v>
       </c>
       <c r="B69">
@@ -1597,14 +1547,14 @@
         <v>25114</v>
       </c>
       <c r="D69">
-        <v>1.4545454545454641E-2</v>
+        <v>0.01454545454545464</v>
       </c>
       <c r="E69">
-        <v>1.5076189321369339E-2</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="2">
+        <v>0.01507618932136934</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5">
+      <c r="A70" s="1">
         <v>45915</v>
       </c>
       <c r="B70">
@@ -1614,14 +1564,14 @@
         <v>25327.05078125</v>
       </c>
       <c r="D70">
-        <v>8.8889063900090548E-3</v>
+        <v>0.008888906390009055</v>
       </c>
       <c r="E70">
-        <v>8.483347186827972E-3</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A71" s="2">
+        <v>0.008483347186827972</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5">
+      <c r="A71" s="1">
         <v>45922</v>
       </c>
       <c r="B71">
@@ -1631,14 +1581,14 @@
         <v>24654.69921875</v>
       </c>
       <c r="D71">
-        <v>-2.117382997810557E-2</v>
+        <v>-0.02117382997810557</v>
       </c>
       <c r="E71">
-        <v>-2.6546776737138011E-2</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="2">
+        <v>-0.02654677673713801</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5">
+      <c r="A72" s="1">
         <v>45929</v>
       </c>
       <c r="B72">
@@ -1648,14 +1598,14 @@
         <v>24894.25</v>
       </c>
       <c r="D72">
-        <v>-1.030774638757914E-2</v>
+        <v>-0.01030774638757914</v>
       </c>
       <c r="E72">
-        <v>9.7162321521173656E-3</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A73" s="2">
+        <v>0.009716232152117366</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5">
+      <c r="A73" s="1">
         <v>45936</v>
       </c>
       <c r="B73">
@@ -1665,14 +1615,14 @@
         <v>25285.349609375</v>
       </c>
       <c r="D73">
-        <v>1.3422272576001371E-2</v>
+        <v>0.01342227257600137</v>
       </c>
       <c r="E73">
-        <v>1.5710439534229789E-2</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A74" s="2">
+        <v>0.01571043953422979</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5">
+      <c r="A74" s="1">
         <v>45943</v>
       </c>
       <c r="B74">
@@ -1682,14 +1632,14 @@
         <v>25709.849609375</v>
       </c>
       <c r="D74">
-        <v>2.5403560032321248E-2</v>
+        <v>0.02540356003232125</v>
       </c>
       <c r="E74">
-        <v>1.6788377719033409E-2</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A75" s="2">
+        <v>0.01678837771903341</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5">
+      <c r="A75" s="1">
         <v>45950</v>
       </c>
       <c r="B75">
@@ -1699,14 +1649,14 @@
         <v>25795.150390625</v>
       </c>
       <c r="D75">
-        <v>2.4562341585600889E-2</v>
+        <v>0.02456234158560089</v>
       </c>
       <c r="E75">
-        <v>3.317824979376605E-3</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A76" s="2">
+        <v>0.003317824979376605</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5">
+      <c r="A76" s="1">
         <v>45957</v>
       </c>
       <c r="B76">
@@ -1716,14 +1666,14 @@
         <v>25722.099609375</v>
       </c>
       <c r="D76">
-        <v>2.3973580472180789E-2</v>
+        <v>0.02397358047218079</v>
       </c>
       <c r="E76">
-        <v>-2.831957951156205E-3</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A77" s="2">
+        <v>-0.002831957951156205</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5">
+      <c r="A77" s="1">
         <v>45964</v>
       </c>
       <c r="B77">
@@ -1733,14 +1683,14 @@
         <v>25492.30078125</v>
       </c>
       <c r="D77">
-        <v>-5.6512542223442486E-3</v>
+        <v>-0.005651254222344249</v>
       </c>
       <c r="E77">
-        <v>-8.9339063146013364E-3</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A78" s="2">
+        <v>-0.008933906314601336</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5">
+      <c r="A78" s="1">
         <v>45971</v>
       </c>
       <c r="B78">
@@ -1750,14 +1700,14 @@
         <v>25910.05078125</v>
       </c>
       <c r="D78">
-        <v>2.7672546964859549E-2</v>
+        <v>0.02767254696485955</v>
       </c>
       <c r="E78">
-        <v>1.638730076130512E-2</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A79" s="2">
+        <v>0.01638730076130512</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5">
+      <c r="A79" s="1">
         <v>45978</v>
       </c>
       <c r="B79">
@@ -1767,14 +1717,14 @@
         <v>26068.150390625</v>
       </c>
       <c r="D79">
-        <v>1.8236849513884709E-2</v>
+        <v>0.01823684951388471</v>
       </c>
       <c r="E79">
-        <v>6.1018641263879134E-3</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A80" s="2">
+        <v>0.006101864126387913</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5">
+      <c r="A80" s="1">
         <v>45985</v>
       </c>
       <c r="B80">
@@ -1784,14 +1734,14 @@
         <v>26202.94921875</v>
       </c>
       <c r="D80">
-        <v>1.3513529512467761E-2</v>
+        <v>0.01351352951246776</v>
       </c>
       <c r="E80">
-        <v>5.1710162057940767E-3</v>
-      </c>
-    </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A81" s="2">
+        <v>0.005171016205794077</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5">
+      <c r="A81" s="1">
         <v>45992</v>
       </c>
       <c r="B81">
@@ -1801,14 +1751,14 @@
         <v>26186.44921875</v>
       </c>
       <c r="D81">
-        <v>-1.7161100104665091E-2</v>
+        <v>-0.01716110010466509</v>
       </c>
       <c r="E81">
-        <v>-6.2970010979501723E-4</v>
-      </c>
-    </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A82" s="2">
+        <v>-0.0006297001097950172</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5">
+      <c r="A82" s="1">
         <v>45999</v>
       </c>
       <c r="B82">
@@ -1818,14 +1768,14 @@
         <v>26046.94921875</v>
       </c>
       <c r="D82">
-        <v>1.032067030120221E-2</v>
+        <v>0.01032067030120221</v>
       </c>
       <c r="E82">
-        <v>-5.3271827285432671E-3</v>
-      </c>
-    </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A83" s="2">
+        <v>-0.005327182728543267</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5">
+      <c r="A83" s="1">
         <v>46006</v>
       </c>
       <c r="B83">
@@ -1835,14 +1785,14 @@
         <v>25966.400390625</v>
       </c>
       <c r="D83">
-        <v>5.5252011474060669E-3</v>
+        <v>0.005525201147406067</v>
       </c>
       <c r="E83">
-        <v>-3.0924476969846899E-3</v>
-      </c>
-    </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A84" s="2">
+        <v>-0.00309244769698469</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5">
+      <c r="A84" s="1">
         <v>46013</v>
       </c>
       <c r="B84">
@@ -1852,14 +1802,14 @@
         <v>26042.30078125</v>
       </c>
       <c r="D84">
-        <v>-3.7697428318300701E-3</v>
+        <v>-0.00376974283183007</v>
       </c>
       <c r="E84">
-        <v>2.9230231947130481E-3</v>
-      </c>
-    </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A85" s="2">
+        <v>0.002923023194713048</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5">
+      <c r="A85" s="1">
         <v>46020</v>
       </c>
       <c r="B85">
@@ -1869,14 +1819,14 @@
         <v>26328.55078125</v>
       </c>
       <c r="D85">
-        <v>2.122889859724042E-2</v>
+        <v>0.02122889859724042</v>
       </c>
       <c r="E85">
-        <v>1.099173235131734E-2</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A86" s="2">
+        <v>0.01099173235131734</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5">
+      <c r="A86" s="1">
         <v>46027</v>
       </c>
       <c r="B86">
@@ -1886,14 +1836,14 @@
         <v>25683.30078125</v>
       </c>
       <c r="D86">
-        <v>-7.3478613585490793E-2</v>
+        <v>-0.07347861358549079</v>
       </c>
       <c r="E86">
-        <v>-2.4507615529659851E-2</v>
-      </c>
-    </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A87" s="2">
+        <v>-0.02450761552965985</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5">
+      <c r="A87" s="1">
         <v>46034</v>
       </c>
       <c r="B87">
@@ -1903,14 +1853,14 @@
         <v>25694.349609375</v>
       </c>
       <c r="D87">
-        <v>-1.179422750503112E-2</v>
+        <v>-0.01179422750503112</v>
       </c>
       <c r="E87">
-        <v>4.3019502123597952E-4</v>
-      </c>
-    </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A88" s="2">
+        <v>0.0004301950212359795</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5">
+      <c r="A88" s="1">
         <v>46041</v>
       </c>
       <c r="B88">
@@ -1920,14 +1870,14 @@
         <v>25048.650390625</v>
       </c>
       <c r="D88">
-        <v>-4.9248952346359842E-2</v>
+        <v>-0.04924895234635984</v>
       </c>
       <c r="E88">
-        <v>-2.51300082923448E-2</v>
-      </c>
-    </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A89" s="2">
+        <v>-0.0251300082923448</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5">
+      <c r="A89" s="1">
         <v>46048</v>
       </c>
       <c r="B89">
@@ -1937,14 +1887,14 @@
         <v>24825.44921875</v>
       </c>
       <c r="D89">
-        <v>-2.8208625838413329E-2</v>
+        <v>-0.02820862583841333</v>
       </c>
       <c r="E89">
-        <v>-8.9107065009194075E-3</v>
-      </c>
-    </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A90" s="2">
+        <v>-0.008910706500919408</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5">
+      <c r="A90" s="1">
         <v>46055</v>
       </c>
       <c r="B90">
@@ -1954,14 +1904,14 @@
         <v>25693.69921875</v>
       </c>
       <c r="D90">
-        <v>7.7060169879825446E-2</v>
+        <v>0.07706016987982545</v>
       </c>
       <c r="E90">
-        <v>3.4974190893763753E-2</v>
-      </c>
-    </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A91" s="2">
+        <v>0.03497419089376375</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5">
+      <c r="A91" s="1">
         <v>46062</v>
       </c>
       <c r="B91">
@@ -1971,14 +1921,14 @@
         <v>25471.099609375</v>
       </c>
       <c r="D91">
-        <v>-2.1505426104299619E-2</v>
+        <v>-0.02150542610429962</v>
       </c>
       <c r="E91">
-        <v>-8.6635874219527231E-3</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A92" s="2">
+        <v>-0.008663587421952723</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5">
+      <c r="A92" s="1">
         <v>46069</v>
       </c>
       <c r="B92">
@@ -1988,14 +1938,14 @@
         <v>25571.25</v>
       </c>
       <c r="D92">
-        <v>-1.4085036299926751E-4</v>
+        <v>-0.0001408503629992675</v>
       </c>
       <c r="E92">
-        <v>3.9319225381277967E-3</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A93" s="2">
+        <v>0.003931922538127797</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5">
+      <c r="A93" s="1">
         <v>46076</v>
       </c>
       <c r="B93">
@@ -2005,14 +1955,14 @@
         <v>25178.650390625</v>
       </c>
       <c r="D93">
-        <v>-1.7965337157526459E-2</v>
+        <v>-0.01796533715752646</v>
       </c>
       <c r="E93">
-        <v>-1.535316456469671E-2</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A94" s="2">
+        <v>-0.01535316456469671</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5">
+      <c r="A94" s="1">
         <v>46083</v>
       </c>
       <c r="B94">
@@ -2022,14 +1972,14 @@
         <v>24450.44921875</v>
       </c>
       <c r="D94">
-        <v>7.8198035893173312E-3</v>
+        <v>0.007819803589317331</v>
       </c>
       <c r="E94">
-        <v>-2.8921374282480872E-2</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A95" s="2">
+        <v>-0.02892137428248087</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5">
+      <c r="A95" s="1">
         <v>46090</v>
       </c>
       <c r="B95">
@@ -2039,14 +1989,14 @@
         <v>23151.099609375</v>
       </c>
       <c r="D95">
-        <v>-1.715553589021734E-2</v>
+        <v>-0.01715553589021734</v>
       </c>
       <c r="E95">
-        <v>-5.3142156929312567E-2</v>
-      </c>
-    </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A96" s="2">
+        <v>-0.05314215692931257</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5">
+      <c r="A96" s="1">
         <v>46097</v>
       </c>
       <c r="B96">
@@ -2056,14 +2006,14 @@
         <v>23114.5</v>
       </c>
       <c r="D96">
-        <v>2.4407962941973341E-2</v>
+        <v>0.02440796294197334</v>
       </c>
       <c r="E96">
-        <v>-1.580901555111369E-3</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A97" s="2">
+        <v>-0.001580901555111369</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5">
+      <c r="A97" s="1">
         <v>46104</v>
       </c>
       <c r="B97">
@@ -2073,14 +2023,14 @@
         <v>22819.599609375</v>
       </c>
       <c r="D97">
-        <v>-4.6875033713033809E-2</v>
+        <v>-0.04687503371303381</v>
       </c>
       <c r="E97">
-        <v>-1.275824225594324E-2</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A98" s="2">
+        <v>-0.01275824225594324</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5">
+      <c r="A98" s="1">
         <v>46111</v>
       </c>
       <c r="B98">
@@ -2090,14 +2040,14 @@
         <v>22713.099609375</v>
       </c>
       <c r="D98">
-        <v>1.780301503988557E-3</v>
+        <v>0.001780301503988557</v>
       </c>
       <c r="E98">
-        <v>-4.6670406940990672E-3</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A99" s="2">
+        <v>-0.004667040694099067</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5">
+      <c r="A99" s="1">
         <v>46118</v>
       </c>
       <c r="B99">
@@ -2107,14 +2057,14 @@
         <v>24050.599609375</v>
       </c>
       <c r="D99">
-        <v>-2.2217610375785399E-4</v>
+        <v>-0.000222176103757854</v>
       </c>
       <c r="E99">
-        <v>5.888672277243634E-2</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A100" s="2">
+        <v>0.05888672277243634</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5">
+      <c r="A100" s="1">
         <v>46125</v>
       </c>
       <c r="B100">
@@ -2124,14 +2074,14 @@
         <v>24353.55078125</v>
       </c>
       <c r="D100">
-        <v>1.096137562090682E-2</v>
+        <v>0.01096137562090682</v>
       </c>
       <c r="E100">
-        <v>1.2596408272370411E-2</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A101" s="2">
+        <v>0.01259640827237041</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5">
+      <c r="A101" s="1">
         <v>46132</v>
       </c>
       <c r="B101">
@@ -2141,14 +2091,14 @@
         <v>23897.94921875</v>
       </c>
       <c r="D101">
-        <v>-2.7252711481227099E-2</v>
+        <v>-0.0272527114812271</v>
       </c>
       <c r="E101">
-        <v>-1.8707808425651451E-2</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A102" s="2">
+        <v>-0.01870780842565145</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5">
+      <c r="A102" s="1">
         <v>46139</v>
       </c>
       <c r="B102">
@@ -2158,14 +2108,14 @@
         <v>23997.55078125</v>
       </c>
       <c r="D102">
-        <v>7.7571920629845303E-2</v>
+        <v>0.0775719206298453</v>
       </c>
       <c r="E102">
-        <v>4.1677870175509391E-3</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A103" s="2">
+        <v>0.004167787017550939</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5">
+      <c r="A103" s="1">
         <v>46146</v>
       </c>
       <c r="B103">
@@ -2175,14 +2125,14 @@
         <v>24176.150390625</v>
       </c>
       <c r="D103">
-        <v>3.0751343259693979E-3</v>
+        <v>0.003075134325969398</v>
       </c>
       <c r="E103">
-        <v>7.442409894369062E-3</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A104" s="2">
+        <v>0.007442409894369062</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5">
+      <c r="A104" s="1">
         <v>46153</v>
       </c>
       <c r="B104">
@@ -2192,10 +2142,10 @@
         <v>23643.5</v>
       </c>
       <c r="D104">
-        <v>-6.8840531019486173E-2</v>
+        <v>-0.06884053101948617</v>
       </c>
       <c r="E104">
-        <v>-2.203205977869627E-2</v>
+        <v>-0.02203205977869627</v>
       </c>
     </row>
   </sheetData>
@@ -2204,25 +2154,25 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4">
+      <c r="A1" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>7</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2233,10 +2183,10 @@
         <v>93500</v>
       </c>
       <c r="D2">
-        <v>83746.586580981733</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+        <v>83746.58658098173</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2247,10 +2197,10 @@
         <v>102850</v>
       </c>
       <c r="D3">
-        <v>82511.656046657299</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+        <v>82511.6560466573</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2261,10 +2211,10 @@
         <v>113135</v>
       </c>
       <c r="D4">
-        <v>81294.935847665547</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+        <v>81294.93584766555</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5">
         <v>4</v>
       </c>
@@ -2275,10 +2225,10 @@
         <v>124448.5000000001</v>
       </c>
       <c r="D5">
-        <v>80096.157453669191</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+        <v>80096.15745366919</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2289,7 +2239,7 @@
         <v>136893.35</v>
       </c>
       <c r="D6">
-        <v>78915.056294090027</v>
+        <v>78915.05629409003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>